<commit_message>
fix(template): correct H14 HH formula and blank stale worker cells
El template venía con H14 apuntando a la fila 29 (chgen) en vez de la 30
(chintegral), y con 6 valores ABRIL obsoletos en las celdas HH de
trabajadores. build() ahora corrige H14 a =H30*0.5 y vacía las 8 celdas HH
de trabajadores antes de guardar; verify() comprueba las fórmulas de HH y
el blanco. Regenera el binario —el diff toca exactamente 7 celdas— y añade
test_template_formulas.py con 16 casos.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/RESUMEN_template_v1.xlsx
+++ b/data/templates/RESUMEN_template_v1.xlsx
@@ -1833,7 +1833,7 @@
       </c>
       <c r="G14" s="41" t="n"/>
       <c r="H14" s="26">
-        <f>H29*0.5</f>
+        <f>H30*0.5</f>
         <v/>
       </c>
       <c r="I14" s="27" t="n"/>
@@ -2578,25 +2578,19 @@
           <t>Cantidad de Trabajadores ch gral</t>
         </is>
       </c>
-      <c r="J29" s="34" t="n">
-        <v>479</v>
-      </c>
+      <c r="J29" s="34" t="n"/>
       <c r="K29" s="31" t="inlineStr">
         <is>
           <t>Cantidad de Trabajadores</t>
         </is>
       </c>
-      <c r="L29" s="34" t="n">
-        <v>5255</v>
-      </c>
+      <c r="L29" s="34" t="n"/>
       <c r="M29" s="31" t="inlineStr">
         <is>
           <t>Cantidad de Trabajadores</t>
         </is>
       </c>
-      <c r="N29" s="38" t="n">
-        <v>4851</v>
-      </c>
+      <c r="N29" s="38" t="n"/>
       <c r="O29" s="69" t="n"/>
     </row>
     <row r="30" customFormat="1" s="52">
@@ -2613,25 +2607,19 @@
           <t>cantidad trab. Ch. integral</t>
         </is>
       </c>
-      <c r="J30" s="52" t="n">
-        <v>123</v>
-      </c>
+      <c r="J30" s="52" t="n"/>
       <c r="K30" s="52" t="inlineStr">
         <is>
           <t>cantidad trab. Ch. integral</t>
         </is>
       </c>
-      <c r="L30" s="69" t="n">
-        <v>373</v>
-      </c>
+      <c r="L30" s="69" t="n"/>
       <c r="M30" s="52" t="inlineStr">
         <is>
           <t>cantidad trab. Ch. integral</t>
         </is>
       </c>
-      <c r="N30" s="69" t="n">
-        <v>784</v>
-      </c>
+      <c r="N30" s="69" t="n"/>
       <c r="O30" s="69" t="n"/>
     </row>
     <row r="31" customFormat="1" s="52">

</xml_diff>

<commit_message>
fix(excel): repair TOTAL Cantidad Realizada O11 #REF! + O12 off-by-one
O11 had lost its K11 ref to #REF! and O12 referenced K11 instead of K12 (odi
summed irl's Río Bueno). Both now SUM(G,I,K,M) for their own row, matching the
rest of the column. Dated backup kept locally (untracked).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/RESUMEN_template_v1.xlsx
+++ b/data/templates/RESUMEN_template_v1.xlsx
@@ -1717,7 +1717,7 @@
         <v/>
       </c>
       <c r="O11" s="19">
-        <f>SUM(G11,I11,#REF!,M11)</f>
+        <f>SUM(G11,I11,K11,M11)</f>
         <v/>
       </c>
       <c r="P11" s="112">
@@ -1762,7 +1762,7 @@
         <v/>
       </c>
       <c r="O12" s="19">
-        <f>SUM(G12,I12,K11,M12)</f>
+        <f>SUM(G12,I12,K12,M12)</f>
         <v/>
       </c>
       <c r="P12" s="112">

</xml_diff>

<commit_message>
fix(cphs): correct CHPS->CPHS in app labels and Excel (display-only)
Visible code/label corrected to the right acronym (Comité Paritario de Higiene y
Seguridad). Internal key 'chps' unchanged (glob/folder/DB/named ranges intact):
SIGLA_LABELS.chps='CPHS', new siglaDisplay() maps the list/header code to 'cphs',
template B31 label and build script updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/RESUMEN_template_v1.xlsx
+++ b/data/templates/RESUMEN_template_v1.xlsx
@@ -1376,7 +1376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:Z36"/>
+  <dimension ref="A1:Z36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.3984375" defaultRowHeight="13.8"/>
   <cols>
     <col width="3.59765625" customWidth="1" style="69" min="1" max="1"/>
@@ -2626,7 +2626,7 @@
       <c r="A31" s="69" t="n"/>
       <c r="B31" s="52" t="inlineStr">
         <is>
-          <t>CHPS — Comité Paritario de Higiene y Seguridad</t>
+          <t>CPHS — Comité Paritario de Higiene y Seguridad</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">

</xml_diff>

<commit_message>
fix(excel): inset logo within header box + match bodega title font
Logo overlapped the header box borders at 110px anchored flush to B2. Re-anchor
at 90px with a OneCellAnchor offset (10px left, 13px top) so it floats inside the
B2:D5 box without touching the black borders. Row 18 (bodegas SUSPEL/RESPEL) title
shipped at Arial 10 while every other category title is Arial 11 — copy B17's font
so the column reads uniformly. Verified via LibreOffice render.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/RESUMEN_template_v1.xlsx
+++ b/data/templates/RESUMEN_template_v1.xlsx
@@ -1060,11 +1060,11 @@
   <oneCellAnchor>
     <from>
       <col>1</col>
-      <colOff>0</colOff>
+      <colOff>95250</colOff>
       <row>1</row>
-      <rowOff>0</rowOff>
+      <rowOff>123825</rowOff>
     </from>
-    <ext cx="1047750" cy="1047750"/>
+    <ext cx="857250" cy="857250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2031,7 +2031,7 @@
     </row>
     <row r="18" customFormat="1" s="52">
       <c r="A18" s="69" t="n"/>
-      <c r="B18" s="65" t="inlineStr">
+      <c r="B18" s="59" t="inlineStr">
         <is>
           <t>N° de Inspecciones a bodegas SUSPEL/RESPEL</t>
         </is>

</xml_diff>

<commit_message>
style(excel): tidy report layout (header width, far-right borders, CPHS row)
Polish reported on the MAYO export, all coordinate-safe (named ranges in B..P
untouched, so downstream consumers are unaffected):

- The title merge spanned E2:Z5 and every data row carried borders out to column Z,
  while the data table ends at P -> a stray "right border" far past the table.
  Narrow the header/band merges (E2:P5, B6:P7, B8:P8) and clear borders + fills in
  the empty Q:Z columns so the box ends at the table edge.
- CPHS (row 31) shipped in Aptos Narrow with no borders; restyle it from a category
  row (row 28) so it reads as part of the list. It stays at row 31 (coordinates +
  named ranges intact), per the chosen "reformat in place" option.

Verified via LibreOffice render against the live MAYO session.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/RESUMEN_template_v1.xlsx
+++ b/data/templates/RESUMEN_template_v1.xlsx
@@ -185,7 +185,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="44">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -728,6 +728,7 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -736,7 +737,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1042,6 +1043,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1078,6 +1086,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1406,7 +1417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:Z36"/>
+  <dimension ref="A1:Z36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.3984375" defaultRowHeight="13.8"/>
   <cols>
     <col width="3.59765625" customWidth="1" style="69" min="1" max="1"/>
@@ -1437,7 +1448,18 @@
     <col width="11.3984375" customWidth="1" style="36" min="27" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.4" customHeight="1" thickBot="1"/>
+    <row r="1" ht="14.4" customHeight="1" thickBot="1">
+      <c r="Q1" s="117" t="n"/>
+      <c r="R1" s="117" t="n"/>
+      <c r="S1" s="117" t="n"/>
+      <c r="T1" s="117" t="n"/>
+      <c r="U1" s="117" t="n"/>
+      <c r="V1" s="117" t="n"/>
+      <c r="W1" s="117" t="n"/>
+      <c r="X1" s="117" t="n"/>
+      <c r="Y1" s="117" t="n"/>
+      <c r="Z1" s="117" t="n"/>
+    </row>
     <row r="2" ht="21.75" customHeight="1">
       <c r="B2" s="93" t="n"/>
       <c r="C2" s="94" t="n"/>
@@ -1459,27 +1481,47 @@
       <c r="M2" s="94" t="n"/>
       <c r="N2" s="94" t="n"/>
       <c r="O2" s="94" t="n"/>
-      <c r="P2" s="94" t="n"/>
-      <c r="Q2" s="94" t="n"/>
-      <c r="R2" s="94" t="n"/>
-      <c r="S2" s="94" t="n"/>
-      <c r="T2" s="94" t="n"/>
-      <c r="U2" s="94" t="n"/>
-      <c r="V2" s="94" t="n"/>
-      <c r="W2" s="94" t="n"/>
-      <c r="X2" s="94" t="n"/>
-      <c r="Y2" s="94" t="n"/>
-      <c r="Z2" s="96" t="n"/>
+      <c r="P2" s="96" t="n"/>
+      <c r="Q2" s="117" t="n"/>
+      <c r="R2" s="117" t="n"/>
+      <c r="S2" s="117" t="n"/>
+      <c r="T2" s="117" t="n"/>
+      <c r="U2" s="117" t="n"/>
+      <c r="V2" s="117" t="n"/>
+      <c r="W2" s="117" t="n"/>
+      <c r="X2" s="117" t="n"/>
+      <c r="Y2" s="117" t="n"/>
+      <c r="Z2" s="117" t="n"/>
     </row>
     <row r="3" ht="21.75" customHeight="1">
       <c r="B3" s="97" t="n"/>
       <c r="E3" s="97" t="n"/>
-      <c r="Z3" s="98" t="n"/>
+      <c r="P3" s="98" t="n"/>
+      <c r="Q3" s="117" t="n"/>
+      <c r="R3" s="117" t="n"/>
+      <c r="S3" s="117" t="n"/>
+      <c r="T3" s="117" t="n"/>
+      <c r="U3" s="117" t="n"/>
+      <c r="V3" s="117" t="n"/>
+      <c r="W3" s="117" t="n"/>
+      <c r="X3" s="117" t="n"/>
+      <c r="Y3" s="117" t="n"/>
+      <c r="Z3" s="117" t="n"/>
     </row>
     <row r="4" ht="21.75" customHeight="1">
       <c r="B4" s="97" t="n"/>
       <c r="E4" s="97" t="n"/>
-      <c r="Z4" s="98" t="n"/>
+      <c r="P4" s="98" t="n"/>
+      <c r="Q4" s="117" t="n"/>
+      <c r="R4" s="117" t="n"/>
+      <c r="S4" s="117" t="n"/>
+      <c r="T4" s="117" t="n"/>
+      <c r="U4" s="117" t="n"/>
+      <c r="V4" s="117" t="n"/>
+      <c r="W4" s="117" t="n"/>
+      <c r="X4" s="117" t="n"/>
+      <c r="Y4" s="117" t="n"/>
+      <c r="Z4" s="117" t="n"/>
     </row>
     <row r="5" ht="21.75" customHeight="1" thickBot="1">
       <c r="B5" s="99" t="n"/>
@@ -1496,17 +1538,17 @@
       <c r="M5" s="100" t="n"/>
       <c r="N5" s="100" t="n"/>
       <c r="O5" s="100" t="n"/>
-      <c r="P5" s="100" t="n"/>
-      <c r="Q5" s="100" t="n"/>
-      <c r="R5" s="100" t="n"/>
-      <c r="S5" s="100" t="n"/>
-      <c r="T5" s="100" t="n"/>
-      <c r="U5" s="100" t="n"/>
-      <c r="V5" s="100" t="n"/>
-      <c r="W5" s="100" t="n"/>
-      <c r="X5" s="100" t="n"/>
-      <c r="Y5" s="100" t="n"/>
-      <c r="Z5" s="101" t="n"/>
+      <c r="P5" s="101" t="n"/>
+      <c r="Q5" s="117" t="n"/>
+      <c r="R5" s="117" t="n"/>
+      <c r="S5" s="117" t="n"/>
+      <c r="T5" s="117" t="n"/>
+      <c r="U5" s="117" t="n"/>
+      <c r="V5" s="117" t="n"/>
+      <c r="W5" s="117" t="n"/>
+      <c r="X5" s="117" t="n"/>
+      <c r="Y5" s="117" t="n"/>
+      <c r="Z5" s="117" t="n"/>
     </row>
     <row r="6" ht="14.7" customHeight="1">
       <c r="B6" s="102" t="inlineStr">
@@ -1527,17 +1569,17 @@
       <c r="M6" s="94" t="n"/>
       <c r="N6" s="94" t="n"/>
       <c r="O6" s="94" t="n"/>
-      <c r="P6" s="94" t="n"/>
-      <c r="Q6" s="94" t="n"/>
-      <c r="R6" s="94" t="n"/>
-      <c r="S6" s="94" t="n"/>
-      <c r="T6" s="103" t="n"/>
-      <c r="U6" s="36" t="n"/>
-      <c r="V6" s="36" t="n"/>
-      <c r="W6" s="36" t="n"/>
-      <c r="X6" s="36" t="n"/>
-      <c r="Y6" s="36" t="n"/>
-      <c r="Z6" s="37" t="n"/>
+      <c r="P6" s="103" t="n"/>
+      <c r="Q6" s="117" t="n"/>
+      <c r="R6" s="117" t="n"/>
+      <c r="S6" s="117" t="n"/>
+      <c r="T6" s="117" t="n"/>
+      <c r="U6" s="118" t="n"/>
+      <c r="V6" s="118" t="n"/>
+      <c r="W6" s="118" t="n"/>
+      <c r="X6" s="118" t="n"/>
+      <c r="Y6" s="118" t="n"/>
+      <c r="Z6" s="118" t="n"/>
     </row>
     <row r="7" ht="14.7" customHeight="1" thickBot="1">
       <c r="B7" s="99" t="n"/>
@@ -1554,17 +1596,17 @@
       <c r="M7" s="100" t="n"/>
       <c r="N7" s="100" t="n"/>
       <c r="O7" s="100" t="n"/>
-      <c r="P7" s="100" t="n"/>
-      <c r="Q7" s="100" t="n"/>
-      <c r="R7" s="100" t="n"/>
-      <c r="S7" s="100" t="n"/>
-      <c r="T7" s="104" t="n"/>
-      <c r="U7" s="36" t="n"/>
-      <c r="V7" s="36" t="n"/>
-      <c r="W7" s="36" t="n"/>
-      <c r="X7" s="36" t="n"/>
-      <c r="Y7" s="36" t="n"/>
-      <c r="Z7" s="37" t="n"/>
+      <c r="P7" s="104" t="n"/>
+      <c r="Q7" s="117" t="n"/>
+      <c r="R7" s="117" t="n"/>
+      <c r="S7" s="117" t="n"/>
+      <c r="T7" s="117" t="n"/>
+      <c r="U7" s="118" t="n"/>
+      <c r="V7" s="118" t="n"/>
+      <c r="W7" s="118" t="n"/>
+      <c r="X7" s="118" t="n"/>
+      <c r="Y7" s="118" t="n"/>
+      <c r="Z7" s="118" t="n"/>
     </row>
     <row r="8" ht="14.4" customHeight="1" thickBot="1">
       <c r="B8" s="66" t="n"/>
@@ -1582,11 +1624,16 @@
       <c r="N8" s="94" t="n"/>
       <c r="O8" s="94" t="n"/>
       <c r="P8" s="94" t="n"/>
-      <c r="Q8" s="94" t="n"/>
-      <c r="R8" s="94" t="n"/>
-      <c r="S8" s="94" t="n"/>
-      <c r="T8" s="94" t="n"/>
-      <c r="Z8" s="3" t="n"/>
+      <c r="Q8" s="117" t="n"/>
+      <c r="R8" s="117" t="n"/>
+      <c r="S8" s="117" t="n"/>
+      <c r="T8" s="117" t="n"/>
+      <c r="U8" s="117" t="n"/>
+      <c r="V8" s="117" t="n"/>
+      <c r="W8" s="117" t="n"/>
+      <c r="X8" s="117" t="n"/>
+      <c r="Y8" s="117" t="n"/>
+      <c r="Z8" s="118" t="n"/>
     </row>
     <row r="9" ht="28.2" customHeight="1" thickBot="1">
       <c r="B9" s="90" t="inlineStr">
@@ -1662,7 +1709,16 @@
 HH Capacitación</t>
         </is>
       </c>
-      <c r="Z9" s="3" t="n"/>
+      <c r="Q9" s="117" t="n"/>
+      <c r="R9" s="117" t="n"/>
+      <c r="S9" s="117" t="n"/>
+      <c r="T9" s="117" t="n"/>
+      <c r="U9" s="117" t="n"/>
+      <c r="V9" s="117" t="n"/>
+      <c r="W9" s="117" t="n"/>
+      <c r="X9" s="117" t="n"/>
+      <c r="Y9" s="117" t="n"/>
+      <c r="Z9" s="118" t="n"/>
     </row>
     <row r="10" customFormat="1" s="52">
       <c r="A10" s="69" t="n"/>
@@ -1707,7 +1763,16 @@
         <f>SUM(N10,L10,J10,H10)</f>
         <v/>
       </c>
-      <c r="Z10" s="14" t="n"/>
+      <c r="Q10" s="117" t="n"/>
+      <c r="R10" s="117" t="n"/>
+      <c r="S10" s="117" t="n"/>
+      <c r="T10" s="117" t="n"/>
+      <c r="U10" s="117" t="n"/>
+      <c r="V10" s="117" t="n"/>
+      <c r="W10" s="117" t="n"/>
+      <c r="X10" s="117" t="n"/>
+      <c r="Y10" s="117" t="n"/>
+      <c r="Z10" s="119" t="n"/>
     </row>
     <row r="11" customFormat="1" s="52">
       <c r="A11" s="69" t="n"/>
@@ -1752,7 +1817,16 @@
         <f>SUM(N11,L11,J11,H11)</f>
         <v/>
       </c>
-      <c r="Z11" s="14" t="n"/>
+      <c r="Q11" s="117" t="n"/>
+      <c r="R11" s="117" t="n"/>
+      <c r="S11" s="117" t="n"/>
+      <c r="T11" s="117" t="n"/>
+      <c r="U11" s="117" t="n"/>
+      <c r="V11" s="117" t="n"/>
+      <c r="W11" s="117" t="n"/>
+      <c r="X11" s="117" t="n"/>
+      <c r="Y11" s="117" t="n"/>
+      <c r="Z11" s="119" t="n"/>
     </row>
     <row r="12" customFormat="1" s="52">
       <c r="A12" s="69" t="n"/>
@@ -1797,7 +1871,16 @@
         <f>SUM(N12,L12,J12,H12)</f>
         <v/>
       </c>
-      <c r="Z12" s="14" t="n"/>
+      <c r="Q12" s="117" t="n"/>
+      <c r="R12" s="117" t="n"/>
+      <c r="S12" s="117" t="n"/>
+      <c r="T12" s="117" t="n"/>
+      <c r="U12" s="117" t="n"/>
+      <c r="V12" s="117" t="n"/>
+      <c r="W12" s="117" t="n"/>
+      <c r="X12" s="117" t="n"/>
+      <c r="Y12" s="117" t="n"/>
+      <c r="Z12" s="119" t="n"/>
     </row>
     <row r="13" customFormat="1" s="52">
       <c r="A13" s="69" t="n"/>
@@ -1842,7 +1925,16 @@
         <f>SUM(N13,L13,J13,H13)</f>
         <v/>
       </c>
-      <c r="Z13" s="14" t="n"/>
+      <c r="Q13" s="117" t="n"/>
+      <c r="R13" s="117" t="n"/>
+      <c r="S13" s="117" t="n"/>
+      <c r="T13" s="117" t="n"/>
+      <c r="U13" s="117" t="n"/>
+      <c r="V13" s="117" t="n"/>
+      <c r="W13" s="117" t="n"/>
+      <c r="X13" s="117" t="n"/>
+      <c r="Y13" s="117" t="n"/>
+      <c r="Z13" s="119" t="n"/>
     </row>
     <row r="14" customFormat="1" s="52">
       <c r="A14" s="69" t="n"/>
@@ -1887,7 +1979,16 @@
         <f>SUM(N14,L14,J14,H14)</f>
         <v/>
       </c>
-      <c r="Z14" s="14" t="n"/>
+      <c r="Q14" s="117" t="n"/>
+      <c r="R14" s="117" t="n"/>
+      <c r="S14" s="117" t="n"/>
+      <c r="T14" s="117" t="n"/>
+      <c r="U14" s="117" t="n"/>
+      <c r="V14" s="117" t="n"/>
+      <c r="W14" s="117" t="n"/>
+      <c r="X14" s="117" t="n"/>
+      <c r="Y14" s="117" t="n"/>
+      <c r="Z14" s="119" t="n"/>
     </row>
     <row r="15" customFormat="1" s="52">
       <c r="A15" s="69" t="n"/>
@@ -1932,7 +2033,16 @@
         <f>SUM(N15,L15,J15,H15)</f>
         <v/>
       </c>
-      <c r="Z15" s="14" t="n"/>
+      <c r="Q15" s="117" t="n"/>
+      <c r="R15" s="117" t="n"/>
+      <c r="S15" s="117" t="n"/>
+      <c r="T15" s="117" t="n"/>
+      <c r="U15" s="117" t="n"/>
+      <c r="V15" s="117" t="n"/>
+      <c r="W15" s="117" t="n"/>
+      <c r="X15" s="117" t="n"/>
+      <c r="Y15" s="117" t="n"/>
+      <c r="Z15" s="119" t="n"/>
     </row>
     <row r="16" customFormat="1" s="52">
       <c r="A16" s="69" t="n"/>
@@ -1977,7 +2087,16 @@
         <f>SUM(N16,L16,J16,H16)</f>
         <v/>
       </c>
-      <c r="Z16" s="14" t="n"/>
+      <c r="Q16" s="117" t="n"/>
+      <c r="R16" s="117" t="n"/>
+      <c r="S16" s="117" t="n"/>
+      <c r="T16" s="117" t="n"/>
+      <c r="U16" s="117" t="n"/>
+      <c r="V16" s="117" t="n"/>
+      <c r="W16" s="117" t="n"/>
+      <c r="X16" s="117" t="n"/>
+      <c r="Y16" s="117" t="n"/>
+      <c r="Z16" s="119" t="n"/>
     </row>
     <row r="17" customFormat="1" s="52">
       <c r="A17" s="69" t="n"/>
@@ -2027,7 +2146,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z17" s="14" t="n"/>
+      <c r="Q17" s="117" t="n"/>
+      <c r="R17" s="117" t="n"/>
+      <c r="S17" s="117" t="n"/>
+      <c r="T17" s="117" t="n"/>
+      <c r="U17" s="117" t="n"/>
+      <c r="V17" s="117" t="n"/>
+      <c r="W17" s="117" t="n"/>
+      <c r="X17" s="117" t="n"/>
+      <c r="Y17" s="117" t="n"/>
+      <c r="Z17" s="119" t="n"/>
     </row>
     <row r="18" customFormat="1" s="52">
       <c r="A18" s="69" t="n"/>
@@ -2077,7 +2205,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z18" s="14" t="n"/>
+      <c r="Q18" s="117" t="n"/>
+      <c r="R18" s="117" t="n"/>
+      <c r="S18" s="117" t="n"/>
+      <c r="T18" s="117" t="n"/>
+      <c r="U18" s="117" t="n"/>
+      <c r="V18" s="117" t="n"/>
+      <c r="W18" s="117" t="n"/>
+      <c r="X18" s="117" t="n"/>
+      <c r="Y18" s="117" t="n"/>
+      <c r="Z18" s="119" t="n"/>
     </row>
     <row r="19" customFormat="1" s="52">
       <c r="A19" s="69" t="n"/>
@@ -2127,7 +2264,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z19" s="14" t="n"/>
+      <c r="Q19" s="117" t="n"/>
+      <c r="R19" s="117" t="n"/>
+      <c r="S19" s="117" t="n"/>
+      <c r="T19" s="117" t="n"/>
+      <c r="U19" s="117" t="n"/>
+      <c r="V19" s="117" t="n"/>
+      <c r="W19" s="117" t="n"/>
+      <c r="X19" s="117" t="n"/>
+      <c r="Y19" s="117" t="n"/>
+      <c r="Z19" s="119" t="n"/>
     </row>
     <row r="20" customFormat="1" s="52">
       <c r="A20" s="69" t="n"/>
@@ -2177,7 +2323,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z20" s="14" t="n"/>
+      <c r="Q20" s="117" t="n"/>
+      <c r="R20" s="117" t="n"/>
+      <c r="S20" s="117" t="n"/>
+      <c r="T20" s="117" t="n"/>
+      <c r="U20" s="117" t="n"/>
+      <c r="V20" s="117" t="n"/>
+      <c r="W20" s="117" t="n"/>
+      <c r="X20" s="117" t="n"/>
+      <c r="Y20" s="117" t="n"/>
+      <c r="Z20" s="119" t="n"/>
     </row>
     <row r="21" customFormat="1" s="52">
       <c r="A21" s="69" t="n"/>
@@ -2227,7 +2382,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z21" s="14" t="n"/>
+      <c r="Q21" s="117" t="n"/>
+      <c r="R21" s="117" t="n"/>
+      <c r="S21" s="117" t="n"/>
+      <c r="T21" s="117" t="n"/>
+      <c r="U21" s="117" t="n"/>
+      <c r="V21" s="117" t="n"/>
+      <c r="W21" s="117" t="n"/>
+      <c r="X21" s="117" t="n"/>
+      <c r="Y21" s="117" t="n"/>
+      <c r="Z21" s="119" t="n"/>
     </row>
     <row r="22" customFormat="1" s="52">
       <c r="A22" s="69" t="n"/>
@@ -2285,7 +2449,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z22" s="14" t="n"/>
+      <c r="Q22" s="117" t="n"/>
+      <c r="R22" s="117" t="n"/>
+      <c r="S22" s="117" t="n"/>
+      <c r="T22" s="117" t="n"/>
+      <c r="U22" s="117" t="n"/>
+      <c r="V22" s="117" t="n"/>
+      <c r="W22" s="117" t="n"/>
+      <c r="X22" s="117" t="n"/>
+      <c r="Y22" s="117" t="n"/>
+      <c r="Z22" s="119" t="n"/>
     </row>
     <row r="23" customFormat="1" s="52">
       <c r="A23" s="69" t="n"/>
@@ -2335,7 +2508,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z23" s="14" t="n"/>
+      <c r="Q23" s="117" t="n"/>
+      <c r="R23" s="117" t="n"/>
+      <c r="S23" s="117" t="n"/>
+      <c r="T23" s="117" t="n"/>
+      <c r="U23" s="117" t="n"/>
+      <c r="V23" s="117" t="n"/>
+      <c r="W23" s="117" t="n"/>
+      <c r="X23" s="117" t="n"/>
+      <c r="Y23" s="117" t="n"/>
+      <c r="Z23" s="119" t="n"/>
     </row>
     <row r="24" customFormat="1" s="52">
       <c r="A24" s="69" t="n"/>
@@ -2385,7 +2567,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z24" s="14" t="n"/>
+      <c r="Q24" s="117" t="n"/>
+      <c r="R24" s="117" t="n"/>
+      <c r="S24" s="117" t="n"/>
+      <c r="T24" s="117" t="n"/>
+      <c r="U24" s="117" t="n"/>
+      <c r="V24" s="117" t="n"/>
+      <c r="W24" s="117" t="n"/>
+      <c r="X24" s="117" t="n"/>
+      <c r="Y24" s="117" t="n"/>
+      <c r="Z24" s="119" t="n"/>
     </row>
     <row r="25" customFormat="1" s="52">
       <c r="A25" s="69" t="n"/>
@@ -2435,7 +2626,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z25" s="14" t="n"/>
+      <c r="Q25" s="117" t="n"/>
+      <c r="R25" s="117" t="n"/>
+      <c r="S25" s="117" t="n"/>
+      <c r="T25" s="117" t="n"/>
+      <c r="U25" s="117" t="n"/>
+      <c r="V25" s="117" t="n"/>
+      <c r="W25" s="117" t="n"/>
+      <c r="X25" s="117" t="n"/>
+      <c r="Y25" s="117" t="n"/>
+      <c r="Z25" s="119" t="n"/>
     </row>
     <row r="26" customFormat="1" s="52">
       <c r="A26" s="69" t="n"/>
@@ -2493,7 +2693,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z26" s="14" t="n"/>
+      <c r="Q26" s="117" t="n"/>
+      <c r="R26" s="117" t="n"/>
+      <c r="S26" s="117" t="n"/>
+      <c r="T26" s="117" t="n"/>
+      <c r="U26" s="117" t="n"/>
+      <c r="V26" s="117" t="n"/>
+      <c r="W26" s="117" t="n"/>
+      <c r="X26" s="117" t="n"/>
+      <c r="Y26" s="117" t="n"/>
+      <c r="Z26" s="119" t="n"/>
     </row>
     <row r="27" customFormat="1" s="52">
       <c r="A27" s="69" t="n"/>
@@ -2543,7 +2752,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z27" s="14" t="n"/>
+      <c r="Q27" s="117" t="n"/>
+      <c r="R27" s="117" t="n"/>
+      <c r="S27" s="117" t="n"/>
+      <c r="T27" s="117" t="n"/>
+      <c r="U27" s="117" t="n"/>
+      <c r="V27" s="117" t="n"/>
+      <c r="W27" s="117" t="n"/>
+      <c r="X27" s="117" t="n"/>
+      <c r="Y27" s="117" t="n"/>
+      <c r="Z27" s="119" t="n"/>
     </row>
     <row r="28" ht="14.4" customFormat="1" customHeight="1" s="52" thickBot="1">
       <c r="A28" s="69" t="n"/>
@@ -2593,7 +2811,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="Z28" s="14" t="n"/>
+      <c r="Q28" s="117" t="n"/>
+      <c r="R28" s="117" t="n"/>
+      <c r="S28" s="117" t="n"/>
+      <c r="T28" s="117" t="n"/>
+      <c r="U28" s="117" t="n"/>
+      <c r="V28" s="117" t="n"/>
+      <c r="W28" s="117" t="n"/>
+      <c r="X28" s="117" t="n"/>
+      <c r="Y28" s="117" t="n"/>
+      <c r="Z28" s="119" t="n"/>
     </row>
     <row r="29" ht="14.4" customFormat="1" customHeight="1" s="52" thickBot="1">
       <c r="A29" s="69" t="n"/>
@@ -2628,6 +2855,16 @@
       </c>
       <c r="N29" s="38" t="n"/>
       <c r="O29" s="69" t="n"/>
+      <c r="Q29" s="117" t="n"/>
+      <c r="R29" s="117" t="n"/>
+      <c r="S29" s="117" t="n"/>
+      <c r="T29" s="117" t="n"/>
+      <c r="U29" s="117" t="n"/>
+      <c r="V29" s="117" t="n"/>
+      <c r="W29" s="117" t="n"/>
+      <c r="X29" s="117" t="n"/>
+      <c r="Y29" s="117" t="n"/>
+      <c r="Z29" s="117" t="n"/>
     </row>
     <row r="30" customFormat="1" s="52">
       <c r="A30" s="69" t="n"/>
@@ -2657,53 +2894,137 @@
       </c>
       <c r="N30" s="69" t="n"/>
       <c r="O30" s="69" t="n"/>
+      <c r="Q30" s="117" t="n"/>
+      <c r="R30" s="117" t="n"/>
+      <c r="S30" s="117" t="n"/>
+      <c r="T30" s="117" t="n"/>
+      <c r="U30" s="117" t="n"/>
+      <c r="V30" s="117" t="n"/>
+      <c r="W30" s="117" t="n"/>
+      <c r="X30" s="117" t="n"/>
+      <c r="Y30" s="117" t="n"/>
+      <c r="Z30" s="117" t="n"/>
     </row>
     <row r="31" customFormat="1" s="52">
       <c r="A31" s="69" t="n"/>
-      <c r="B31" s="52" t="inlineStr">
+      <c r="B31" s="53" t="inlineStr">
         <is>
           <t>CPHS — Comité Paritario de Higiene y Seguridad</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="C31" s="120" t="n"/>
+      <c r="D31" s="120" t="n"/>
+      <c r="E31" s="121" t="n"/>
+      <c r="F31" s="40" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O31" s="69" t="n"/>
+      <c r="G31" s="45" t="n"/>
+      <c r="H31" s="16" t="n"/>
+      <c r="I31" s="29" t="n"/>
+      <c r="J31" s="16" t="n"/>
+      <c r="K31" s="29" t="n"/>
+      <c r="L31" s="16" t="n"/>
+      <c r="M31" s="25" t="n"/>
+      <c r="N31" s="16" t="n"/>
+      <c r="O31" s="23" t="n"/>
+      <c r="P31" s="24" t="n"/>
+      <c r="Q31" s="117" t="n"/>
+      <c r="R31" s="117" t="n"/>
+      <c r="S31" s="117" t="n"/>
+      <c r="T31" s="117" t="n"/>
+      <c r="U31" s="117" t="n"/>
+      <c r="V31" s="117" t="n"/>
+      <c r="W31" s="117" t="n"/>
+      <c r="X31" s="117" t="n"/>
+      <c r="Y31" s="117" t="n"/>
+      <c r="Z31" s="117" t="n"/>
     </row>
     <row r="32" customFormat="1" s="52">
       <c r="A32" s="69" t="n"/>
       <c r="B32" s="52" t="n"/>
       <c r="O32" s="69" t="n"/>
+      <c r="Q32" s="117" t="n"/>
+      <c r="R32" s="117" t="n"/>
+      <c r="S32" s="117" t="n"/>
+      <c r="T32" s="117" t="n"/>
+      <c r="U32" s="117" t="n"/>
+      <c r="V32" s="117" t="n"/>
+      <c r="W32" s="117" t="n"/>
+      <c r="X32" s="117" t="n"/>
+      <c r="Y32" s="117" t="n"/>
+      <c r="Z32" s="117" t="n"/>
     </row>
     <row r="33" customFormat="1" s="52">
       <c r="A33" s="69" t="n"/>
       <c r="B33" s="52" t="n"/>
       <c r="O33" s="69" t="n"/>
+      <c r="Q33" s="117" t="n"/>
+      <c r="R33" s="117" t="n"/>
+      <c r="S33" s="117" t="n"/>
+      <c r="T33" s="117" t="n"/>
+      <c r="U33" s="117" t="n"/>
+      <c r="V33" s="117" t="n"/>
+      <c r="W33" s="117" t="n"/>
+      <c r="X33" s="117" t="n"/>
+      <c r="Y33" s="117" t="n"/>
+      <c r="Z33" s="117" t="n"/>
     </row>
     <row r="34" customFormat="1" s="52">
       <c r="A34" s="69" t="n"/>
       <c r="B34" s="52" t="n"/>
       <c r="O34" s="69" t="n"/>
+      <c r="Q34" s="117" t="n"/>
+      <c r="R34" s="117" t="n"/>
+      <c r="S34" s="117" t="n"/>
+      <c r="T34" s="117" t="n"/>
+      <c r="U34" s="117" t="n"/>
+      <c r="V34" s="117" t="n"/>
+      <c r="W34" s="117" t="n"/>
+      <c r="X34" s="117" t="n"/>
+      <c r="Y34" s="117" t="n"/>
+      <c r="Z34" s="117" t="n"/>
     </row>
     <row r="35" customFormat="1" s="52">
       <c r="A35" s="69" t="n"/>
       <c r="B35" s="52" t="n"/>
       <c r="O35" s="69" t="n"/>
+      <c r="Q35" s="117" t="n"/>
+      <c r="R35" s="117" t="n"/>
+      <c r="S35" s="117" t="n"/>
+      <c r="T35" s="117" t="n"/>
+      <c r="U35" s="117" t="n"/>
+      <c r="V35" s="117" t="n"/>
+      <c r="W35" s="117" t="n"/>
+      <c r="X35" s="117" t="n"/>
+      <c r="Y35" s="117" t="n"/>
+      <c r="Z35" s="117" t="n"/>
     </row>
     <row r="36" customFormat="1" s="52">
       <c r="A36" s="69" t="n"/>
       <c r="B36" s="52" t="n"/>
       <c r="O36" s="69" t="n"/>
+      <c r="Q36" s="117" t="n"/>
+      <c r="R36" s="117" t="n"/>
+      <c r="S36" s="117" t="n"/>
+      <c r="T36" s="117" t="n"/>
+      <c r="U36" s="117" t="n"/>
+      <c r="V36" s="117" t="n"/>
+      <c r="W36" s="117" t="n"/>
+      <c r="X36" s="117" t="n"/>
+      <c r="Y36" s="117" t="n"/>
+      <c r="Z36" s="117" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="E2:P5"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B8:P8"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="B36:E36"/>
     <mergeCell ref="B32:E32"/>
@@ -2717,15 +3038,13 @@
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B2:D5"/>
     <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B6:T7"/>
     <mergeCell ref="B21:E21"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="B14:E14"/>
-    <mergeCell ref="E2:Z5"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B8:T8"/>
     <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B6:P7"/>
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="B34:E34"/>

</xml_diff>

<commit_message>
feat(excel): dynamic report title (month/year) instead of hardcoded MARZO 2026
The template's E2 shipped a static "RESUMEN EJECUTIVO…\nMARZO 2026\nPROYECTO RED
LOS RÍOS - LOS LAGOS", so every month's RESUMEN read "MARZO 2026" regardless of the
session. Add a `report_title` named range -> E2 and have the output route compute
the title from the session's year/month (project line stays constant). Verified via
LibreOffice render: a 2026-05 export now reads "MAYO 2026".

Tests: _build_report_title unit cases + an end-to-end check that the generated
title cell shows the session month and not MARZO.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/RESUMEN_template_v1.xlsx
+++ b/data/templates/RESUMEN_template_v1.xlsx
@@ -89,6 +89,7 @@
     <definedName name="HRB_workers_chintegral">'Cump. Programa Prevención'!$L$30</definedName>
     <definedName name="HPV_workers_chgen">'Cump. Programa Prevención'!$N$29</definedName>
     <definedName name="HPV_workers_chintegral">'Cump. Programa Prevención'!$N$30</definedName>
+    <definedName name="report_title">'Cump. Programa Prevención'!$E$2</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -195,7 +196,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="54">
+  <borders count="64">
     <border>
       <left/>
       <right/>
@@ -792,6 +793,76 @@
       <right style="medium"/>
       <top style="thin"/>
       <bottom style="medium"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="medium"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="medium"/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="5">
@@ -801,7 +872,7 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1200,6 +1271,12 @@
     <xf numFmtId="4" fontId="6" fillId="2" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1791,9 +1868,9 @@
           <t>Cumplimiento Operacional</t>
         </is>
       </c>
-      <c r="C9" s="123" t="n"/>
-      <c r="D9" s="123" t="n"/>
-      <c r="E9" s="123" t="n"/>
+      <c r="C9" s="154" t="n"/>
+      <c r="D9" s="154" t="n"/>
+      <c r="E9" s="155" t="n"/>
       <c r="F9" s="124" t="inlineStr">
         <is>
           <t xml:space="preserve">Periodicidad de acuerdo a Plan de Prevención </t>
@@ -1877,9 +1954,9 @@
           <t>N° de Reuniones de Prevención de Riesgos</t>
         </is>
       </c>
-      <c r="C10" s="131" t="n"/>
-      <c r="D10" s="131" t="n"/>
-      <c r="E10" s="131" t="n"/>
+      <c r="C10" s="156" t="n"/>
+      <c r="D10" s="156" t="n"/>
+      <c r="E10" s="157" t="n"/>
       <c r="F10" s="132" t="inlineStr">
         <is>
           <t>Mensual</t>
@@ -1931,9 +2008,9 @@
           <t>N° de Charlas de Inducción (ODI)</t>
         </is>
       </c>
-      <c r="C11" s="131" t="n"/>
-      <c r="D11" s="131" t="n"/>
-      <c r="E11" s="131" t="n"/>
+      <c r="C11" s="156" t="n"/>
+      <c r="D11" s="156" t="n"/>
+      <c r="E11" s="157" t="n"/>
       <c r="F11" s="132" t="inlineStr">
         <is>
           <t>Cada vez</t>
@@ -1985,9 +2062,9 @@
           <t>N° de Charlas de Inducción Visita</t>
         </is>
       </c>
-      <c r="C12" s="131" t="n"/>
-      <c r="D12" s="131" t="n"/>
-      <c r="E12" s="131" t="n"/>
+      <c r="C12" s="156" t="n"/>
+      <c r="D12" s="156" t="n"/>
+      <c r="E12" s="157" t="n"/>
       <c r="F12" s="132" t="inlineStr">
         <is>
           <t>Cada vez</t>
@@ -2039,9 +2116,9 @@
           <t>N° de Charlas Generales (Diarias)</t>
         </is>
       </c>
-      <c r="C13" s="131" t="n"/>
-      <c r="D13" s="131" t="n"/>
-      <c r="E13" s="131" t="n"/>
+      <c r="C13" s="156" t="n"/>
+      <c r="D13" s="156" t="n"/>
+      <c r="E13" s="157" t="n"/>
       <c r="F13" s="132" t="inlineStr">
         <is>
           <t>Diaria</t>
@@ -2093,9 +2170,9 @@
           <t>N° de Charlas Integrales</t>
         </is>
       </c>
-      <c r="C14" s="131" t="n"/>
-      <c r="D14" s="131" t="n"/>
-      <c r="E14" s="131" t="n"/>
+      <c r="C14" s="156" t="n"/>
+      <c r="D14" s="156" t="n"/>
+      <c r="E14" s="157" t="n"/>
       <c r="F14" s="132" t="inlineStr">
         <is>
           <t>Semanal</t>
@@ -2147,9 +2224,9 @@
           <t>Difusión de PTS</t>
         </is>
       </c>
-      <c r="C15" s="131" t="n"/>
-      <c r="D15" s="131" t="n"/>
-      <c r="E15" s="131" t="n"/>
+      <c r="C15" s="156" t="n"/>
+      <c r="D15" s="156" t="n"/>
+      <c r="E15" s="157" t="n"/>
       <c r="F15" s="132" t="inlineStr">
         <is>
           <t>Cada vez</t>
@@ -2201,9 +2278,9 @@
           <t>ART realizadas</t>
         </is>
       </c>
-      <c r="C16" s="131" t="n"/>
-      <c r="D16" s="131" t="n"/>
-      <c r="E16" s="131" t="n"/>
+      <c r="C16" s="156" t="n"/>
+      <c r="D16" s="156" t="n"/>
+      <c r="E16" s="157" t="n"/>
       <c r="F16" s="132" t="inlineStr">
         <is>
           <t>Diaria</t>
@@ -2255,9 +2332,9 @@
           <t>N° de Inspecciones Generales a las áreas de trabajo</t>
         </is>
       </c>
-      <c r="C17" s="131" t="n"/>
-      <c r="D17" s="131" t="n"/>
-      <c r="E17" s="131" t="n"/>
+      <c r="C17" s="156" t="n"/>
+      <c r="D17" s="156" t="n"/>
+      <c r="E17" s="157" t="n"/>
       <c r="F17" s="132" t="inlineStr">
         <is>
           <t>Mensual</t>
@@ -2314,9 +2391,9 @@
           <t>N° de Inspecciones a bodegas SUSPEL/RESPEL</t>
         </is>
       </c>
-      <c r="C18" s="131" t="n"/>
-      <c r="D18" s="131" t="n"/>
-      <c r="E18" s="131" t="n"/>
+      <c r="C18" s="156" t="n"/>
+      <c r="D18" s="156" t="n"/>
+      <c r="E18" s="157" t="n"/>
       <c r="F18" s="132" t="inlineStr">
         <is>
           <t>Trimestral</t>
@@ -2373,9 +2450,9 @@
           <t>N° de Inspecciones a maquinarias y equipo</t>
         </is>
       </c>
-      <c r="C19" s="131" t="n"/>
-      <c r="D19" s="131" t="n"/>
-      <c r="E19" s="131" t="n"/>
+      <c r="C19" s="156" t="n"/>
+      <c r="D19" s="156" t="n"/>
+      <c r="E19" s="157" t="n"/>
       <c r="F19" s="132" t="inlineStr">
         <is>
           <t>Diaria</t>
@@ -2432,9 +2509,9 @@
           <t>N° de Inspecciones a equipamiento de emergencia (extintores)</t>
         </is>
       </c>
-      <c r="C20" s="131" t="n"/>
-      <c r="D20" s="131" t="n"/>
-      <c r="E20" s="131" t="n"/>
+      <c r="C20" s="156" t="n"/>
+      <c r="D20" s="156" t="n"/>
+      <c r="E20" s="157" t="n"/>
       <c r="F20" s="132" t="inlineStr">
         <is>
           <t>Mensual</t>
@@ -2491,9 +2568,9 @@
           <t>N° de Inspecciones a señalética de obra</t>
         </is>
       </c>
-      <c r="C21" s="131" t="n"/>
-      <c r="D21" s="131" t="n"/>
-      <c r="E21" s="131" t="n"/>
+      <c r="C21" s="156" t="n"/>
+      <c r="D21" s="156" t="n"/>
+      <c r="E21" s="157" t="n"/>
       <c r="F21" s="132" t="inlineStr">
         <is>
           <t>Trimestral</t>
@@ -2550,9 +2627,9 @@
           <t>Revisión de Documentación de maquinaria</t>
         </is>
       </c>
-      <c r="C22" s="131" t="n"/>
-      <c r="D22" s="131" t="n"/>
-      <c r="E22" s="131" t="n"/>
+      <c r="C22" s="156" t="n"/>
+      <c r="D22" s="156" t="n"/>
+      <c r="E22" s="157" t="n"/>
       <c r="F22" s="132" t="inlineStr">
         <is>
           <t>Mensual</t>
@@ -2617,9 +2694,9 @@
           <t>Inspección de medidas de seguridad en excavaciones</t>
         </is>
       </c>
-      <c r="C23" s="131" t="n"/>
-      <c r="D23" s="131" t="n"/>
-      <c r="E23" s="131" t="n"/>
+      <c r="C23" s="156" t="n"/>
+      <c r="D23" s="156" t="n"/>
+      <c r="E23" s="157" t="n"/>
       <c r="F23" s="132" t="inlineStr">
         <is>
           <t>Mensual</t>
@@ -2676,9 +2753,9 @@
           <t>Inspección a medidas de seguridad en trabajo en altura</t>
         </is>
       </c>
-      <c r="C24" s="131" t="n"/>
-      <c r="D24" s="131" t="n"/>
-      <c r="E24" s="131" t="n"/>
+      <c r="C24" s="156" t="n"/>
+      <c r="D24" s="156" t="n"/>
+      <c r="E24" s="157" t="n"/>
       <c r="F24" s="132" t="inlineStr">
         <is>
           <t>Semanal</t>
@@ -2735,9 +2812,9 @@
           <t>Inspección de Medidas de Seguridad para trabajo en caliente.</t>
         </is>
       </c>
-      <c r="C25" s="131" t="n"/>
-      <c r="D25" s="131" t="n"/>
-      <c r="E25" s="131" t="n"/>
+      <c r="C25" s="156" t="n"/>
+      <c r="D25" s="156" t="n"/>
+      <c r="E25" s="157" t="n"/>
       <c r="F25" s="132" t="inlineStr">
         <is>
           <t>Semanal</t>
@@ -2794,9 +2871,9 @@
           <t>Inspección de Medidas de Seguridad para trabajos en espacios confinados.</t>
         </is>
       </c>
-      <c r="C26" s="131" t="n"/>
-      <c r="D26" s="131" t="n"/>
-      <c r="E26" s="131" t="n"/>
+      <c r="C26" s="156" t="n"/>
+      <c r="D26" s="156" t="n"/>
+      <c r="E26" s="157" t="n"/>
       <c r="F26" s="139" t="inlineStr">
         <is>
           <t>Diaria</t>
@@ -2861,9 +2938,9 @@
           <t>Inspección de Herramientas Eléctricas</t>
         </is>
       </c>
-      <c r="C27" s="131" t="n"/>
-      <c r="D27" s="131" t="n"/>
-      <c r="E27" s="131" t="n"/>
+      <c r="C27" s="156" t="n"/>
+      <c r="D27" s="156" t="n"/>
+      <c r="E27" s="157" t="n"/>
       <c r="F27" s="132" t="inlineStr">
         <is>
           <t>Semanal</t>
@@ -2920,9 +2997,9 @@
           <t>Inspección de Andamios</t>
         </is>
       </c>
-      <c r="C28" s="131" t="n"/>
-      <c r="D28" s="131" t="n"/>
-      <c r="E28" s="131" t="n"/>
+      <c r="C28" s="156" t="n"/>
+      <c r="D28" s="156" t="n"/>
+      <c r="E28" s="157" t="n"/>
       <c r="F28" s="132" t="inlineStr">
         <is>
           <t>Diaria</t>
@@ -2979,9 +3056,9 @@
           <t>Cantidad de Trabajadores — Charlas Generales</t>
         </is>
       </c>
-      <c r="C29" s="142" t="n"/>
-      <c r="D29" s="142" t="n"/>
-      <c r="E29" s="142" t="n"/>
+      <c r="C29" s="156" t="n"/>
+      <c r="D29" s="156" t="n"/>
+      <c r="E29" s="157" t="n"/>
       <c r="F29" s="143" t="n"/>
       <c r="G29" s="143" t="n"/>
       <c r="H29" s="144" t="n"/>
@@ -3011,9 +3088,9 @@
           <t>Cantidad de Trabajadores — Charlas Integrales</t>
         </is>
       </c>
-      <c r="C30" s="142" t="n"/>
-      <c r="D30" s="142" t="n"/>
-      <c r="E30" s="142" t="n"/>
+      <c r="C30" s="156" t="n"/>
+      <c r="D30" s="156" t="n"/>
+      <c r="E30" s="157" t="n"/>
       <c r="F30" s="142" t="n"/>
       <c r="G30" s="143" t="n"/>
       <c r="H30" s="144" t="n"/>
@@ -3043,9 +3120,9 @@
           <t>CPHS — Comité Paritario de Higiene y Seguridad</t>
         </is>
       </c>
-      <c r="C31" s="148" t="n"/>
-      <c r="D31" s="148" t="n"/>
-      <c r="E31" s="148" t="n"/>
+      <c r="C31" s="158" t="n"/>
+      <c r="D31" s="158" t="n"/>
+      <c r="E31" s="159" t="n"/>
       <c r="F31" s="149" t="inlineStr">
         <is>
           <t>—</t>

</xml_diff>

<commit_message>
feat(excel): wire HPV dif_pts worker total to N15 (template)
Add named range HPV_workers_difpts -> N15 and clear the =M15*0.5
fallback to 0. The writer overwrites N15 with the counted worker
total; uncounted HPV shows an explicit 0 (Incr 3B, decision D2).
Other hospitals' row-15 HH formulas (H15/J15/L15) untouched.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/RESUMEN_template_v1.xlsx
+++ b/data/templates/RESUMEN_template_v1.xlsx
@@ -90,6 +90,7 @@
     <definedName name="HPV_workers_chgen">'Cump. Programa Prevención'!$N$29</definedName>
     <definedName name="HPV_workers_chintegral">'Cump. Programa Prevención'!$N$30</definedName>
     <definedName name="report_title">'Cump. Programa Prevención'!$E$2</definedName>
+    <definedName name="HPV_workers_difpts">'Cump. Programa Prevención'!$N$15</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -2248,9 +2249,8 @@
         <v/>
       </c>
       <c r="M15" s="133" t="n"/>
-      <c r="N15" s="134">
-        <f>M15*0.5</f>
-        <v/>
+      <c r="N15" s="134" t="n">
+        <v>0</v>
       </c>
       <c r="O15" s="135">
         <f>SUM(G15,I15,K15,M15)</f>

</xml_diff>

<commit_message>
feat(excel): wire revdocmaq->B22 + espacios->B26, drop chps ranges
Direct additive openpyxl edit of the hand-patched template (NOT regenerated):
+8 named ranges (revdocmaq row 22, espacios row 26; G=HLL/I=HLU/K=HRB/M=HPV),
-4 chps ranges. Verified integrity (image 1->1, N15/O11/O12 formulas + dims
unchanged) against a dated backup. 76 count ranges. Builder maps + verify() +
README synced as docs (builder stays non-idempotent, not run).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/RESUMEN_template_v1.xlsx
+++ b/data/templates/RESUMEN_template_v1.xlsx
@@ -77,10 +77,6 @@
     <definedName name="HLU_andamios_count">'Cump. Programa Prevención'!$I$28</definedName>
     <definedName name="HRB_andamios_count">'Cump. Programa Prevención'!$K$28</definedName>
     <definedName name="HPV_andamios_count">'Cump. Programa Prevención'!$M$28</definedName>
-    <definedName name="HLL_chps_count">'Cump. Programa Prevención'!$G$31</definedName>
-    <definedName name="HLU_chps_count">'Cump. Programa Prevención'!$I$31</definedName>
-    <definedName name="HRB_chps_count">'Cump. Programa Prevención'!$K$31</definedName>
-    <definedName name="HPV_chps_count">'Cump. Programa Prevención'!$M$31</definedName>
     <definedName name="HLL_workers_chgen">'Cump. Programa Prevención'!$H$29</definedName>
     <definedName name="HLL_workers_chintegral">'Cump. Programa Prevención'!$H$30</definedName>
     <definedName name="HLU_workers_chgen">'Cump. Programa Prevención'!$J$29</definedName>
@@ -91,6 +87,14 @@
     <definedName name="HPV_workers_chintegral">'Cump. Programa Prevención'!$N$30</definedName>
     <definedName name="report_title">'Cump. Programa Prevención'!$E$2</definedName>
     <definedName name="HPV_workers_difpts">'Cump. Programa Prevención'!$N$15</definedName>
+    <definedName name="HLL_revdocmaq_count">'Cump. Programa Prevención'!$G$22</definedName>
+    <definedName name="HLL_espacios_count">'Cump. Programa Prevención'!$G$26</definedName>
+    <definedName name="HLU_revdocmaq_count">'Cump. Programa Prevención'!$I$22</definedName>
+    <definedName name="HLU_espacios_count">'Cump. Programa Prevención'!$I$26</definedName>
+    <definedName name="HRB_revdocmaq_count">'Cump. Programa Prevención'!$K$22</definedName>
+    <definedName name="HRB_espacios_count">'Cump. Programa Prevención'!$K$26</definedName>
+    <definedName name="HPV_revdocmaq_count">'Cump. Programa Prevención'!$M$22</definedName>
+    <definedName name="HPV_espacios_count">'Cump. Programa Prevención'!$M$26</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>

</xml_diff>